<commit_message>
Agrego flujo de diagrama dentro del mismo excel, en la hoja flujo de diagrama
</commit_message>
<xml_diff>
--- a/Momento 1 Prueba de escritorio y diccionario.xlsx
+++ b/Momento 1 Prueba de escritorio y diccionario.xlsx
@@ -8,13 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/597136a9be4b2f9f/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{0393C76D-9E93-49F8-A689-3D4FD58396D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="8_{0393C76D-9E93-49F8-A689-3D4FD58396D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{40FBBBFF-1F3B-4EC6-B4EC-6842C47726BC}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{76A8FC27-4B89-47D7-BBE8-2B6D78434E8C}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{76A8FC27-4B89-47D7-BBE8-2B6D78434E8C}"/>
   </bookViews>
   <sheets>
     <sheet name="Prueba de Escritorio" sheetId="1" r:id="rId1"/>
     <sheet name="Diccionario" sheetId="2" r:id="rId2"/>
+    <sheet name="Flujograma" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029" iterateDelta="1E-4"/>
   <extLst>
@@ -274,6 +275,2547 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>419100</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>152400</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>297180</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>15240</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="2" name="Elipse 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{2EFF83C5-6F52-2FDC-CC6C-5AEC31666BE8}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3589020" y="701040"/>
+          <a:ext cx="2255520" cy="594360"/>
+        </a:xfrm>
+        <a:prstGeom prst="ellipse">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1">
+            <a:shade val="50000"/>
+          </a:schemeClr>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:endParaRPr lang="es-CO" sz="1100"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>487680</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>129540</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>304800</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>38100</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="3" name="CuadroTexto 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{1B7E21F6-863F-C6E0-1795-F9EC9597104F}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="4450080" y="861060"/>
+          <a:ext cx="609600" cy="274320"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln w="9525" cmpd="sng">
+          <a:solidFill>
+            <a:schemeClr val="lt1">
+              <a:shade val="50000"/>
+            </a:schemeClr>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="es-CO" sz="1100"/>
+            <a:t>INICIO</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>784860</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>45720</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>784860</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>7620</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="5" name="Conector recto de flecha 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{8B88802A-B6AA-1067-D34C-BAA1484E1243}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvCxnSpPr/>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="4747260" y="1325880"/>
+          <a:ext cx="0" cy="510540"/>
+        </a:xfrm>
+        <a:prstGeom prst="straightConnector1">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln>
+          <a:tailEnd type="triangle"/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>30480</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>60960</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>769620</xdr:colOff>
+      <xdr:row>12</xdr:row>
+      <xdr:rowOff>129540</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="11" name="Rectángulo: esquinas redondeadas 10">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{75DDDFE9-4F28-41E2-B067-27399663858C}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3200400" y="1889760"/>
+          <a:ext cx="3116580" cy="434340"/>
+        </a:xfrm>
+        <a:prstGeom prst="roundRect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="accent4">
+            <a:lumMod val="40000"/>
+            <a:lumOff val="60000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1">
+            <a:shade val="50000"/>
+          </a:schemeClr>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:endParaRPr lang="es-CO" sz="1100"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>68580</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>137160</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>739140</xdr:colOff>
+      <xdr:row>12</xdr:row>
+      <xdr:rowOff>45720</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="13" name="CuadroTexto 12">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{0DF60B85-831C-4976-9213-18137F81EF4F}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3238500" y="1965960"/>
+          <a:ext cx="3048000" cy="274320"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln w="9525" cmpd="sng">
+          <a:solidFill>
+            <a:schemeClr val="lt1">
+              <a:shade val="50000"/>
+            </a:schemeClr>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="es-CO" sz="1100"/>
+            <a:t>Leer</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="es-CO" sz="1100" baseline="0"/>
+            <a:t> nombreProducto</a:t>
+          </a:r>
+          <a:endParaRPr lang="es-CO" sz="1100"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>30480</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>45720</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>769620</xdr:colOff>
+      <xdr:row>18</xdr:row>
+      <xdr:rowOff>114300</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="14" name="Rectángulo: esquinas redondeadas 13">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{62C9F861-FDCE-42DE-8EE1-580EA6D4525C}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3200400" y="2971800"/>
+          <a:ext cx="3116580" cy="434340"/>
+        </a:xfrm>
+        <a:prstGeom prst="roundRect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="accent4">
+            <a:lumMod val="40000"/>
+            <a:lumOff val="60000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1">
+            <a:shade val="50000"/>
+          </a:schemeClr>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:endParaRPr lang="es-CO" sz="1100"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>68580</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>121920</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>739140</xdr:colOff>
+      <xdr:row>18</xdr:row>
+      <xdr:rowOff>30480</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="15" name="CuadroTexto 14">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{1AEEDC85-DAF3-420C-9DD6-983518CF46DD}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3238500" y="3048000"/>
+          <a:ext cx="3048000" cy="274320"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln w="9525" cmpd="sng">
+          <a:solidFill>
+            <a:schemeClr val="lt1">
+              <a:shade val="50000"/>
+            </a:schemeClr>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="es-CO" sz="1100"/>
+            <a:t>Leer</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="es-CO" sz="1100" baseline="0"/>
+            <a:t> costoBase</a:t>
+          </a:r>
+          <a:endParaRPr lang="es-CO" sz="1100"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>784860</xdr:colOff>
+      <xdr:row>12</xdr:row>
+      <xdr:rowOff>167640</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>784860</xdr:colOff>
+      <xdr:row>15</xdr:row>
+      <xdr:rowOff>129540</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="18" name="Conector recto de flecha 17">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{CC7749B7-0748-4E32-A0A4-9E917E97E0F3}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvCxnSpPr/>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="4747260" y="2362200"/>
+          <a:ext cx="0" cy="510540"/>
+        </a:xfrm>
+        <a:prstGeom prst="straightConnector1">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln>
+          <a:tailEnd type="triangle"/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>19</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>144780</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="19" name="Conector recto de flecha 18">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{63652FDC-AA94-4F3D-BF06-9EF9265A8ECE}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvCxnSpPr/>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="4754880" y="3474720"/>
+          <a:ext cx="0" cy="510540"/>
+        </a:xfrm>
+        <a:prstGeom prst="straightConnector1">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln>
+          <a:tailEnd type="triangle"/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>30480</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>45720</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>769620</xdr:colOff>
+      <xdr:row>24</xdr:row>
+      <xdr:rowOff>114300</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="20" name="Rectángulo: esquinas redondeadas 19">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{38996F62-A631-4E77-922D-9328BEB411E2}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3200400" y="4069080"/>
+          <a:ext cx="3116580" cy="434340"/>
+        </a:xfrm>
+        <a:prstGeom prst="roundRect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="accent4">
+            <a:lumMod val="40000"/>
+            <a:lumOff val="60000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1">
+            <a:shade val="50000"/>
+          </a:schemeClr>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:endParaRPr lang="es-CO" sz="1100"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>68580</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>121920</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>739140</xdr:colOff>
+      <xdr:row>24</xdr:row>
+      <xdr:rowOff>30480</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="21" name="CuadroTexto 20">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{EDDAEDBC-FEF5-4DB9-A536-D4B5402E5647}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3238500" y="4145280"/>
+          <a:ext cx="3048000" cy="274320"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln w="9525" cmpd="sng">
+          <a:solidFill>
+            <a:schemeClr val="lt1">
+              <a:shade val="50000"/>
+            </a:schemeClr>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="es-CO" sz="1100"/>
+            <a:t>Leer</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="es-CO" sz="1100" baseline="0"/>
+            <a:t> porcentajeGanancia</a:t>
+          </a:r>
+          <a:endParaRPr lang="es-CO" sz="1100"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>25</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>27</xdr:row>
+      <xdr:rowOff>144780</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="22" name="Conector recto de flecha 21">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{05372543-D77D-411E-A2A0-C70749FB95B9}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvCxnSpPr/>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="4754880" y="4572000"/>
+          <a:ext cx="0" cy="510540"/>
+        </a:xfrm>
+        <a:prstGeom prst="straightConnector1">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln>
+          <a:tailEnd type="triangle"/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>7620</xdr:colOff>
+      <xdr:row>28</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>784860</xdr:colOff>
+      <xdr:row>30</xdr:row>
+      <xdr:rowOff>114300</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="23" name="Rectángulo 22">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C18DDA67-36E4-F343-C6BC-5D5116898E07}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3177540" y="5120640"/>
+          <a:ext cx="3154680" cy="480060"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="accent3">
+            <a:lumMod val="40000"/>
+            <a:lumOff val="60000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1">
+            <a:shade val="50000"/>
+          </a:schemeClr>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:endParaRPr lang="es-CO" sz="1100"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>60960</xdr:colOff>
+      <xdr:row>28</xdr:row>
+      <xdr:rowOff>76200</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>731520</xdr:colOff>
+      <xdr:row>30</xdr:row>
+      <xdr:rowOff>38100</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="26" name="CuadroTexto 25">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{1383068B-8A0C-4015-BC0B-7645D5F26B68}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3230880" y="5196840"/>
+          <a:ext cx="3048000" cy="327660"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln w="9525" cmpd="sng">
+          <a:solidFill>
+            <a:schemeClr val="lt1">
+              <a:shade val="50000"/>
+            </a:schemeClr>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="es-CO" sz="1100"/>
+            <a:t>valorGanancia</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="es-CO" sz="1100" baseline="0"/>
+            <a:t> &lt;- costoBase * porcentajeGanancia</a:t>
+          </a:r>
+          <a:endParaRPr lang="es-CO" sz="1100"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>31</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>33</xdr:row>
+      <xdr:rowOff>144780</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="27" name="Conector recto de flecha 26">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{2481D5EA-4A5F-488B-8500-37CD6B418CAA}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvCxnSpPr/>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="4754880" y="5669280"/>
+          <a:ext cx="0" cy="510540"/>
+        </a:xfrm>
+        <a:prstGeom prst="straightConnector1">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln>
+          <a:tailEnd type="triangle"/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>15240</xdr:colOff>
+      <xdr:row>34</xdr:row>
+      <xdr:rowOff>15240</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>36</xdr:row>
+      <xdr:rowOff>129540</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="28" name="Rectángulo 27">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{7B55AC28-1CC8-48BA-A385-0733CE191150}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3185160" y="6233160"/>
+          <a:ext cx="3154680" cy="480060"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="accent3">
+            <a:lumMod val="40000"/>
+            <a:lumOff val="60000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1">
+            <a:shade val="50000"/>
+          </a:schemeClr>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:endParaRPr lang="es-CO" sz="1100"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>68580</xdr:colOff>
+      <xdr:row>34</xdr:row>
+      <xdr:rowOff>91440</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>739140</xdr:colOff>
+      <xdr:row>36</xdr:row>
+      <xdr:rowOff>53340</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="29" name="CuadroTexto 28">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{905D5080-0292-47D9-B6D8-B2EAE63D47E8}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3238500" y="6309360"/>
+          <a:ext cx="3048000" cy="327660"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln w="9525" cmpd="sng">
+          <a:solidFill>
+            <a:schemeClr val="lt1">
+              <a:shade val="50000"/>
+            </a:schemeClr>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="es-CO" sz="1100" baseline="0"/>
+            <a:t>subtotal &lt;- costoBase + valorGanancia</a:t>
+          </a:r>
+          <a:endParaRPr lang="es-CO" sz="1100"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>37</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>39</xdr:row>
+      <xdr:rowOff>144780</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="30" name="Conector recto de flecha 29">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{44D705C8-C0FC-4E18-A5ED-0872F2C96772}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvCxnSpPr/>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="4754880" y="6766560"/>
+          <a:ext cx="0" cy="510540"/>
+        </a:xfrm>
+        <a:prstGeom prst="straightConnector1">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln>
+          <a:tailEnd type="triangle"/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>15240</xdr:colOff>
+      <xdr:row>40</xdr:row>
+      <xdr:rowOff>15240</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>42</xdr:row>
+      <xdr:rowOff>129540</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="31" name="Rectángulo 30">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{74159092-43F0-4C53-B413-4C14432C0EE5}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3185160" y="7330440"/>
+          <a:ext cx="3154680" cy="480060"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="accent3">
+            <a:lumMod val="40000"/>
+            <a:lumOff val="60000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1">
+            <a:shade val="50000"/>
+          </a:schemeClr>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:endParaRPr lang="es-CO" sz="1100"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>68580</xdr:colOff>
+      <xdr:row>40</xdr:row>
+      <xdr:rowOff>91440</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>739140</xdr:colOff>
+      <xdr:row>42</xdr:row>
+      <xdr:rowOff>53340</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="32" name="CuadroTexto 31">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D5B7D04D-4FFA-4CC3-95F0-C4E16823BAB1}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3238500" y="7406640"/>
+          <a:ext cx="3048000" cy="327660"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln w="9525" cmpd="sng">
+          <a:solidFill>
+            <a:schemeClr val="lt1">
+              <a:shade val="50000"/>
+            </a:schemeClr>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="es-CO" sz="1100" baseline="0"/>
+            <a:t>impuestoIVA &lt;- subtotal * IVA</a:t>
+          </a:r>
+          <a:endParaRPr lang="es-CO" sz="1100"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>43</xdr:row>
+      <xdr:rowOff>7620</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>45</xdr:row>
+      <xdr:rowOff>152400</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="33" name="Conector recto de flecha 32">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{8A5AC472-DCC5-4DB0-847D-697C7D104A23}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvCxnSpPr/>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="4754880" y="7871460"/>
+          <a:ext cx="0" cy="510540"/>
+        </a:xfrm>
+        <a:prstGeom prst="straightConnector1">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln>
+          <a:tailEnd type="triangle"/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>7620</xdr:colOff>
+      <xdr:row>46</xdr:row>
+      <xdr:rowOff>22860</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>784860</xdr:colOff>
+      <xdr:row>48</xdr:row>
+      <xdr:rowOff>137160</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="34" name="Rectángulo 33">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{A9F022DB-51C3-4B46-AB33-20CBA44CB6B1}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3177540" y="8435340"/>
+          <a:ext cx="3154680" cy="480060"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="accent3">
+            <a:lumMod val="40000"/>
+            <a:lumOff val="60000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1">
+            <a:shade val="50000"/>
+          </a:schemeClr>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:endParaRPr lang="es-CO" sz="1100"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>60960</xdr:colOff>
+      <xdr:row>46</xdr:row>
+      <xdr:rowOff>99060</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>731520</xdr:colOff>
+      <xdr:row>48</xdr:row>
+      <xdr:rowOff>60960</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="35" name="CuadroTexto 34">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B6BD8D1A-5BBD-46FD-897E-CDE9EBF76059}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3230880" y="8511540"/>
+          <a:ext cx="3048000" cy="327660"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln w="9525" cmpd="sng">
+          <a:solidFill>
+            <a:schemeClr val="lt1">
+              <a:shade val="50000"/>
+            </a:schemeClr>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="es-CO" sz="1100" baseline="0"/>
+            <a:t>precioFinal &lt;- subtotal + impuestoIVA</a:t>
+          </a:r>
+          <a:endParaRPr lang="es-CO" sz="1100"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>49</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>51</xdr:row>
+      <xdr:rowOff>144780</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="36" name="Conector recto de flecha 35">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{48636E22-A6DD-4880-A01B-60E074902666}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvCxnSpPr/>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="4754880" y="8961120"/>
+          <a:ext cx="0" cy="510540"/>
+        </a:xfrm>
+        <a:prstGeom prst="straightConnector1">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln>
+          <a:tailEnd type="triangle"/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>30480</xdr:colOff>
+      <xdr:row>52</xdr:row>
+      <xdr:rowOff>15240</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>769620</xdr:colOff>
+      <xdr:row>54</xdr:row>
+      <xdr:rowOff>83820</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="37" name="Rectángulo: esquinas redondeadas 36">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{A4B23F3B-ECFC-42CE-B6FF-C2BC4BC82872}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3200400" y="9525000"/>
+          <a:ext cx="3116580" cy="434340"/>
+        </a:xfrm>
+        <a:prstGeom prst="roundRect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="accent4">
+            <a:lumMod val="40000"/>
+            <a:lumOff val="60000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1">
+            <a:shade val="50000"/>
+          </a:schemeClr>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:endParaRPr lang="es-CO" sz="1100"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>68580</xdr:colOff>
+      <xdr:row>52</xdr:row>
+      <xdr:rowOff>91440</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>739140</xdr:colOff>
+      <xdr:row>54</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="38" name="CuadroTexto 37">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{051ADAF0-9B8A-4F10-833F-284DD7B8B140}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3238500" y="9601200"/>
+          <a:ext cx="3048000" cy="274320"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln w="9525" cmpd="sng">
+          <a:solidFill>
+            <a:schemeClr val="lt1">
+              <a:shade val="50000"/>
+            </a:schemeClr>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="es-CO" sz="1100"/>
+            <a:t>Escribir</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="es-CO" sz="1100" baseline="0"/>
+            <a:t> valorGanancia</a:t>
+          </a:r>
+          <a:endParaRPr lang="es-CO" sz="1100"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>54</xdr:row>
+      <xdr:rowOff>144780</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>57</xdr:row>
+      <xdr:rowOff>106680</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="39" name="Conector recto de flecha 38">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{157E727C-2894-4A84-BE88-E71A607E6684}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvCxnSpPr/>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="4754880" y="10020300"/>
+          <a:ext cx="0" cy="510540"/>
+        </a:xfrm>
+        <a:prstGeom prst="straightConnector1">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln>
+          <a:tailEnd type="triangle"/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>30480</xdr:colOff>
+      <xdr:row>57</xdr:row>
+      <xdr:rowOff>160020</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>769620</xdr:colOff>
+      <xdr:row>60</xdr:row>
+      <xdr:rowOff>45720</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="40" name="Rectángulo: esquinas redondeadas 39">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C9D7347E-8091-4895-BCB2-73C076C594AF}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3200400" y="10584180"/>
+          <a:ext cx="3116580" cy="434340"/>
+        </a:xfrm>
+        <a:prstGeom prst="roundRect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="accent4">
+            <a:lumMod val="40000"/>
+            <a:lumOff val="60000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1">
+            <a:shade val="50000"/>
+          </a:schemeClr>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:endParaRPr lang="es-CO" sz="1100"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>68580</xdr:colOff>
+      <xdr:row>58</xdr:row>
+      <xdr:rowOff>53340</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>739140</xdr:colOff>
+      <xdr:row>59</xdr:row>
+      <xdr:rowOff>144780</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="41" name="CuadroTexto 40">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{15E92ED6-4E1F-4139-9687-08A4A4C714B0}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3238500" y="10660380"/>
+          <a:ext cx="3048000" cy="274320"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln w="9525" cmpd="sng">
+          <a:solidFill>
+            <a:schemeClr val="lt1">
+              <a:shade val="50000"/>
+            </a:schemeClr>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr marL="0" marR="0" lvl="0" indent="0" algn="ctr" defTabSz="914400" eaLnBrk="1" fontAlgn="auto" latinLnBrk="0" hangingPunct="1">
+            <a:lnSpc>
+              <a:spcPct val="100000"/>
+            </a:lnSpc>
+            <a:spcBef>
+              <a:spcPts val="0"/>
+            </a:spcBef>
+            <a:spcAft>
+              <a:spcPts val="0"/>
+            </a:spcAft>
+            <a:buClrTx/>
+            <a:buSzTx/>
+            <a:buFontTx/>
+            <a:buNone/>
+            <a:tabLst/>
+            <a:defRPr/>
+          </a:pPr>
+          <a:r>
+            <a:rPr lang="es-CO" sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>Escribir</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="es-CO" sz="1100" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t> subtotal</a:t>
+          </a:r>
+          <a:endParaRPr lang="es-CO">
+            <a:effectLst/>
+          </a:endParaRPr>
+        </a:p>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:endParaRPr lang="es-CO" sz="1100"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>60</xdr:row>
+      <xdr:rowOff>91440</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>63</xdr:row>
+      <xdr:rowOff>53340</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="42" name="Conector recto de flecha 41">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{7A292F78-9507-4E75-BC5B-5EC8DD346DEF}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvCxnSpPr/>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="4754880" y="11064240"/>
+          <a:ext cx="0" cy="510540"/>
+        </a:xfrm>
+        <a:prstGeom prst="straightConnector1">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln>
+          <a:tailEnd type="triangle"/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>30480</xdr:colOff>
+      <xdr:row>63</xdr:row>
+      <xdr:rowOff>106680</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>769620</xdr:colOff>
+      <xdr:row>65</xdr:row>
+      <xdr:rowOff>175260</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="43" name="Rectángulo: esquinas redondeadas 42">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{52AD510C-BCCE-4873-8707-F559924499DD}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3200400" y="11628120"/>
+          <a:ext cx="3116580" cy="434340"/>
+        </a:xfrm>
+        <a:prstGeom prst="roundRect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="accent4">
+            <a:lumMod val="40000"/>
+            <a:lumOff val="60000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1">
+            <a:shade val="50000"/>
+          </a:schemeClr>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:endParaRPr lang="es-CO" sz="1100"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>68580</xdr:colOff>
+      <xdr:row>64</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>739140</xdr:colOff>
+      <xdr:row>65</xdr:row>
+      <xdr:rowOff>91440</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="44" name="CuadroTexto 43">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C30C9FA3-9E53-439C-BC95-7C6E8C2B2FF5}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3238500" y="11704320"/>
+          <a:ext cx="3048000" cy="274320"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln w="9525" cmpd="sng">
+          <a:solidFill>
+            <a:schemeClr val="lt1">
+              <a:shade val="50000"/>
+            </a:schemeClr>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr marL="0" marR="0" lvl="0" indent="0" algn="ctr" defTabSz="914400" eaLnBrk="1" fontAlgn="auto" latinLnBrk="0" hangingPunct="1">
+            <a:lnSpc>
+              <a:spcPct val="100000"/>
+            </a:lnSpc>
+            <a:spcBef>
+              <a:spcPts val="0"/>
+            </a:spcBef>
+            <a:spcAft>
+              <a:spcPts val="0"/>
+            </a:spcAft>
+            <a:buClrTx/>
+            <a:buSzTx/>
+            <a:buFontTx/>
+            <a:buNone/>
+            <a:tabLst/>
+            <a:defRPr/>
+          </a:pPr>
+          <a:r>
+            <a:rPr lang="es-CO" sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>Escribir</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="es-CO" sz="1100" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t> impuestoIVA</a:t>
+          </a:r>
+          <a:endParaRPr lang="es-CO">
+            <a:effectLst/>
+          </a:endParaRPr>
+        </a:p>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:endParaRPr lang="es-CO" sz="1100"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>66</xdr:row>
+      <xdr:rowOff>38100</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>69</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="45" name="Conector recto de flecha 44">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{08ED8EDF-740D-4C59-A1DF-6D9C2F7EFFCE}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvCxnSpPr/>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="4754880" y="12108180"/>
+          <a:ext cx="0" cy="510540"/>
+        </a:xfrm>
+        <a:prstGeom prst="straightConnector1">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln>
+          <a:tailEnd type="triangle"/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>30480</xdr:colOff>
+      <xdr:row>69</xdr:row>
+      <xdr:rowOff>53340</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>769620</xdr:colOff>
+      <xdr:row>71</xdr:row>
+      <xdr:rowOff>121920</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="46" name="Rectángulo: esquinas redondeadas 45">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B5305B03-FE8A-4B00-ACE1-B54B3A346558}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3200400" y="12672060"/>
+          <a:ext cx="3116580" cy="434340"/>
+        </a:xfrm>
+        <a:prstGeom prst="roundRect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="accent4">
+            <a:lumMod val="40000"/>
+            <a:lumOff val="60000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1">
+            <a:shade val="50000"/>
+          </a:schemeClr>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:endParaRPr lang="es-CO" sz="1100"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>68580</xdr:colOff>
+      <xdr:row>69</xdr:row>
+      <xdr:rowOff>129540</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>739140</xdr:colOff>
+      <xdr:row>71</xdr:row>
+      <xdr:rowOff>38100</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="47" name="CuadroTexto 46">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{A57C42A7-FD8B-4E50-B335-F620FE78EE0B}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3238500" y="12748260"/>
+          <a:ext cx="3048000" cy="274320"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln w="9525" cmpd="sng">
+          <a:solidFill>
+            <a:schemeClr val="lt1">
+              <a:shade val="50000"/>
+            </a:schemeClr>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr marL="0" marR="0" lvl="0" indent="0" algn="ctr" defTabSz="914400" eaLnBrk="1" fontAlgn="auto" latinLnBrk="0" hangingPunct="1">
+            <a:lnSpc>
+              <a:spcPct val="100000"/>
+            </a:lnSpc>
+            <a:spcBef>
+              <a:spcPts val="0"/>
+            </a:spcBef>
+            <a:spcAft>
+              <a:spcPts val="0"/>
+            </a:spcAft>
+            <a:buClrTx/>
+            <a:buSzTx/>
+            <a:buFontTx/>
+            <a:buNone/>
+            <a:tabLst/>
+            <a:defRPr/>
+          </a:pPr>
+          <a:r>
+            <a:rPr lang="es-CO" sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>Escribir</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="es-CO" sz="1100" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t> precioFinal</a:t>
+          </a:r>
+          <a:endParaRPr lang="es-CO">
+            <a:effectLst/>
+          </a:endParaRPr>
+        </a:p>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:endParaRPr lang="es-CO" sz="1100"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>72</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>74</xdr:row>
+      <xdr:rowOff>144780</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="48" name="Conector recto de flecha 47">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B6A83163-13B0-4CE6-BEAE-E2C453600100}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvCxnSpPr/>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="4754880" y="13167360"/>
+          <a:ext cx="0" cy="510540"/>
+        </a:xfrm>
+        <a:prstGeom prst="straightConnector1">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln>
+          <a:tailEnd type="triangle"/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>457200</xdr:colOff>
+      <xdr:row>75</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>335280</xdr:colOff>
+      <xdr:row>78</xdr:row>
+      <xdr:rowOff>45720</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="49" name="Elipse 48">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D8DD7C76-3B39-409D-9696-A79C92AFD63B}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3627120" y="13716000"/>
+          <a:ext cx="2255520" cy="594360"/>
+        </a:xfrm>
+        <a:prstGeom prst="ellipse">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1">
+            <a:shade val="50000"/>
+          </a:schemeClr>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:endParaRPr lang="es-CO" sz="1100"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>525780</xdr:colOff>
+      <xdr:row>75</xdr:row>
+      <xdr:rowOff>160020</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>342900</xdr:colOff>
+      <xdr:row>77</xdr:row>
+      <xdr:rowOff>68580</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="50" name="CuadroTexto 49">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{FF3A3C3B-31CF-4823-8212-7B8BFA7BE19E}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="4488180" y="13876020"/>
+          <a:ext cx="609600" cy="274320"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln w="9525" cmpd="sng">
+          <a:solidFill>
+            <a:schemeClr val="lt1">
+              <a:shade val="50000"/>
+            </a:schemeClr>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="es-CO" sz="1100"/>
+            <a:t>FIN</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1400,4 +3942,14 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A9EF0375-BD3E-4D28-9D2A-471A79B15F09}">
+  <dimension ref="A1"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>